<commit_message>
added sensitivity analysis and new plot function
</commit_message>
<xml_diff>
--- a/data/input.xlsx
+++ b/data/input.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Google Drive\PycharmProjects\prg-opf\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03730F1E-DD97-4DB9-89BB-47601081A168}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{482BF6CA-B214-404C-A9C6-03B0E7F53806}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="5280" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="5280" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Power Routers" sheetId="1" r:id="rId1"/>
@@ -689,12 +689,6 @@
       <c r="C10" t="s">
         <v>10</v>
       </c>
-      <c r="E10">
-        <v>5</v>
-      </c>
-      <c r="F10">
-        <v>0</v>
-      </c>
       <c r="G10">
         <v>-2.3280000000000001E-5</v>
       </c>

</xml_diff>

<commit_message>
feat: enhance port loss constraints and sensitivity analysis with new input handling
</commit_message>
<xml_diff>
--- a/data/input.xlsx
+++ b/data/input.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Google Drive\PycharmProjects\prg-opf\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{482BF6CA-B214-404C-A9C6-03B0E7F53806}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D03D967-0957-41F9-8424-0FDC4025232B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="5280" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="5280" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Power Routers" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="34">
   <si>
     <t>PR</t>
   </si>
@@ -128,6 +128,9 @@
   </si>
   <si>
     <t>BigM</t>
+  </si>
+  <si>
+    <t>terminal_bus</t>
   </si>
 </sst>
 </file>
@@ -493,6 +496,7 @@
   <dimension ref="A1:H14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="3" max="3" width="12.88671875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -705,6 +709,12 @@
       </c>
       <c r="C11" t="s">
         <v>10</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+      <c r="F11">
+        <v>0</v>
       </c>
       <c r="G11">
         <v>-2.3280000000000001E-5</v>
@@ -774,10 +784,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="3" width="12.33203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>11</v>
       </c>
@@ -785,280 +798,364 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>12</v>
       </c>
       <c r="B2">
         <v>13</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>12</v>
       </c>
       <c r="B3">
         <v>14</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>12</v>
       </c>
       <c r="B4">
         <v>15</v>
       </c>
-      <c r="C4">
+      <c r="C4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D4">
         <v>0.27202871297791642</v>
       </c>
-      <c r="D4">
+      <c r="E4">
         <v>0.1</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>13</v>
       </c>
       <c r="B5">
         <v>16</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>13</v>
       </c>
       <c r="B6">
         <v>17</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>13</v>
       </c>
       <c r="B7">
         <v>18</v>
       </c>
-      <c r="C7">
+      <c r="C7" t="s">
+        <v>33</v>
+      </c>
+      <c r="D7">
         <v>0.27202871297791642</v>
       </c>
-      <c r="D7">
+      <c r="E7">
         <v>0.1</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>14</v>
       </c>
       <c r="B8">
         <v>19</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>14</v>
       </c>
       <c r="B9">
         <v>20</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>14</v>
       </c>
       <c r="B10">
         <v>21</v>
       </c>
-      <c r="C10">
+      <c r="C10" t="s">
+        <v>33</v>
+      </c>
+      <c r="D10">
         <v>0.27202871297791642</v>
       </c>
-      <c r="D10">
+      <c r="E10">
         <v>0.1</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>15</v>
       </c>
       <c r="B11">
         <v>22</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C11" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>15</v>
       </c>
       <c r="B12">
         <v>23</v>
       </c>
-      <c r="C12">
+      <c r="C12" t="s">
+        <v>33</v>
+      </c>
+      <c r="D12">
         <v>0.81608613893374915</v>
       </c>
-      <c r="D12">
+      <c r="E12">
         <v>0.3</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>15</v>
       </c>
       <c r="B13">
         <v>24</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C13" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>16</v>
       </c>
       <c r="B14">
         <v>25</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C14" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>16</v>
       </c>
       <c r="B15">
         <v>26</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C15" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>16</v>
       </c>
       <c r="B16">
         <v>27</v>
       </c>
-      <c r="C16">
+      <c r="C16" t="s">
+        <v>33</v>
+      </c>
+      <c r="D16">
         <v>0.81608613893374915</v>
       </c>
-      <c r="D16">
+      <c r="E16">
         <v>0.3</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>17</v>
       </c>
       <c r="B17">
         <v>28</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C17" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>17</v>
       </c>
       <c r="B18">
         <v>29</v>
       </c>
-      <c r="C18">
-        <v>0</v>
+      <c r="C18" t="s">
+        <v>33</v>
       </c>
       <c r="D18">
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>17</v>
       </c>
       <c r="B19">
         <v>30</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C19" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>18</v>
       </c>
       <c r="B20">
         <v>31</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C20" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>18</v>
       </c>
       <c r="B21">
         <v>32</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C21" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>18</v>
       </c>
       <c r="B22">
         <v>33</v>
       </c>
-      <c r="C22">
+      <c r="C22" t="s">
+        <v>33</v>
+      </c>
+      <c r="D22">
         <v>0.81608613893374915</v>
       </c>
-      <c r="D22">
+      <c r="E22">
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>19</v>
       </c>
       <c r="B23">
         <v>34</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C23" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>19</v>
       </c>
       <c r="B24">
         <v>35</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C24" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>19</v>
       </c>
       <c r="B25">
         <v>36</v>
       </c>
-      <c r="C25">
+      <c r="C25" t="s">
+        <v>33</v>
+      </c>
+      <c r="D25">
         <v>0.81608613893374915</v>
       </c>
-      <c r="D25">
+      <c r="E25">
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>20</v>
       </c>
       <c r="B26">
         <v>37</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C26" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>20</v>
       </c>
       <c r="B27">
         <v>38</v>
       </c>
-      <c r="C27">
+      <c r="C27" t="s">
+        <v>33</v>
+      </c>
+      <c r="D27">
         <v>-0.57991040658668036</v>
       </c>
-      <c r="D27">
+      <c r="E27">
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>20</v>
       </c>
       <c r="B28">
         <v>39</v>
+      </c>
+      <c r="C28" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>